<commit_message>
feat: populate teams and deliverables from excel data dynamically
</commit_message>
<xml_diff>
--- a/docs/ProjectTeams_Details.xlsx
+++ b/docs/ProjectTeams_Details.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nimrita Koul\Documents\3Teaching2022Onwards\Teaching2026_FebtoJune\AgenticAI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nimrita Koul\Documents\3Teaching2022Onwards\Teaching2026_FebtoJune\AgenticAI\AgenticAI_CourseProjects2026\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94732D0A-03A6-4030-A433-B5BE9AE94226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15E6AED2-FCF6-43D3-9F90-22D67087230E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="0" windowWidth="15750" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StudentsList" sheetId="1" r:id="rId1"/>
@@ -597,7 +597,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -638,6 +638,14 @@
       <color rgb="FFFF0000"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -693,7 +701,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -714,9 +722,10 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1876,19 +1885,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="13" t="s">
         <v>126</v>
       </c>
     </row>

</xml_diff>